<commit_message>
Expanded the featurization to include thermodynamic physical descriptors. Results produce TBABH and TMABH melting temperatures that fall within uncertainty of the experimental data.
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D25EFB-A61A-4D24-9091-2882C95C030F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D4E42B-76FE-4822-8401-0C8EB8318DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28455" yWindow="345" windowWidth="21600" windowHeight="14715" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-28110" yWindow="690" windowWidth="21600" windowHeight="14715" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="CATALOG" sheetId="1" r:id="rId1"/>
@@ -1248,7 +1248,7 @@
     <t>Tetraethylammonium Borohydride</t>
   </si>
   <si>
-    <t>[B].CC[N+](CC)(CC)CC</t>
+    <t>CC[N+](CC)(CC)CC.[BH4-]</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Expanding upon melting point prediction capability
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9D4E42B-76FE-4822-8401-0C8EB8318DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF32F9B-D4DF-4480-A69E-4D341762BCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28110" yWindow="690" windowWidth="21600" windowHeight="14715" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-28800" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="CATALOG" sheetId="1" r:id="rId1"/>
@@ -415,7 +415,274 @@
         </r>
       </text>
     </comment>
-    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{74CA7090-F16F-4E81-9C1D-4C76B0CA001F}">
+    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{2CF6CDD1-F5E1-43E8-A19E-28BAAD5C627C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E7" authorId="0" shapeId="0" xr:uid="{67560CD9-4B42-4009-8FEE-B7B0E0D24E47}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{5E82BDD6-5DA8-4D10-AA85-ECD6AB017319}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{471E01A8-C311-4AC7-AEC5-5D6B6CAAD97B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E8" authorId="0" shapeId="0" xr:uid="{CBC558AB-017C-4385-AA76-E249D19B2033}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F8" authorId="0" shapeId="0" xr:uid="{AB8D56E7-0CD8-4253-A680-DB2E9B7966F8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{1E1D85AE-73C9-4EE5-9B10-D99F6D60BD07}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{EB6033F4-CA7E-49DB-BB17-C34560971AF5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{525F711F-3C09-481A-85BF-92F18353722F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=2#Thermo-Condensed</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{E3FE7A1B-338F-492F-A6BF-400F515D6E34}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C112492&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E11" authorId="0" shapeId="0" xr:uid="{65CE4E3C-BF7D-46D6-8CA4-96B3A0D09621}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C112492&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D14" authorId="0" shapeId="0" xr:uid="{B68F36C1-4BA4-48F1-99E3-8AD353A1321A}">
       <text>
         <r>
           <rPr>
@@ -440,251 +707,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D8" authorId="0" shapeId="0" xr:uid="{1E1D85AE-73C9-4EE5-9B10-D99F6D60BD07}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E8" authorId="0" shapeId="0" xr:uid="{EB6033F4-CA7E-49DB-BB17-C34560971AF5}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F8" authorId="0" shapeId="0" xr:uid="{525F711F-3C09-481A-85BF-92F18353722F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C111966&amp;Mask=2#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D9" authorId="0" shapeId="0" xr:uid="{2CF6CDD1-F5E1-43E8-A19E-28BAAD5C627C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E9" authorId="0" shapeId="0" xr:uid="{67560CD9-4B42-4009-8FEE-B7B0E0D24E47}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=4#Thermo-Phase</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F9" authorId="0" shapeId="0" xr:uid="{5E82BDD6-5DA8-4D10-AA85-ECD6AB017319}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-https://webbook.nist.gov/cgi/cbook.cgi?ID=C56815&amp;Units=SI&amp;Mask=2#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D10" authorId="0" shapeId="0" xr:uid="{471E01A8-C311-4AC7-AEC5-5D6B6CAAD97B}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E10" authorId="0" shapeId="0" xr:uid="{CBC558AB-017C-4385-AA76-E249D19B2033}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F10" authorId="0" shapeId="0" xr:uid="{AB8D56E7-0CD8-4253-A680-DB2E9B7966F8}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://webbook.nist.gov/cgi/cbook.cgi?ID=C107153&amp;Mask=1E9F#Thermo-Condensed</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D11" authorId="0" shapeId="0" xr:uid="{B68F36C1-4BA4-48F1-99E3-8AD353A1321A}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://advanced.onlinelibrary.wiley.com/doi/10.1002/adma.202502566</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F11" authorId="0" shapeId="0" xr:uid="{BADEE219-B2DB-4696-8CD3-185AC97E6E32}">
+    <comment ref="F14" authorId="0" shapeId="0" xr:uid="{BADEE219-B2DB-4696-8CD3-185AC97E6E32}">
       <text>
         <r>
           <rPr>
@@ -710,7 +733,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D12" authorId="0" shapeId="0" xr:uid="{63C390B0-F0DD-4E22-8006-4770ED582EEB}">
+    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{63C390B0-F0DD-4E22-8006-4770ED582EEB}">
       <text>
         <r>
           <rPr>
@@ -735,7 +758,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F12" authorId="0" shapeId="0" xr:uid="{E1A1E0C1-3AE1-4CDA-A225-D95E0807710C}">
+    <comment ref="F22" authorId="0" shapeId="0" xr:uid="{E1A1E0C1-3AE1-4CDA-A225-D95E0807710C}">
       <text>
         <r>
           <rPr>
@@ -757,6 +780,31 @@
           <t xml:space="preserve">
 Source(s):
 1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{74CA7090-F16F-4E81-9C1D-4C76B0CA001F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://advanced.onlinelibrary.wiley.com/doi/10.1002/adma.202502566</t>
         </r>
       </text>
     </comment>
@@ -1144,7 +1192,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="74">
   <si>
     <t>Full Name</t>
   </si>
@@ -1215,9 +1263,6 @@
     <t>Tetrabutylammonium Borohydride</t>
   </si>
   <si>
-    <t>[BH4-].CCCC[N+](CCCC)(CCCC)CCCC</t>
-  </si>
-  <si>
     <t>Ammonia Borane</t>
   </si>
   <si>
@@ -1227,9 +1272,6 @@
     <t>Lithium Borohydride</t>
   </si>
   <si>
-    <t>[Li+].[BH4-]</t>
-  </si>
-  <si>
     <t>Sodium Borohydride</t>
   </si>
   <si>
@@ -1249,6 +1291,132 @@
   </si>
   <si>
     <t>CC[N+](CC)(CC)CC.[BH4-]</t>
+  </si>
+  <si>
+    <t>Trigylme</t>
+  </si>
+  <si>
+    <t>Tetraglyme</t>
+  </si>
+  <si>
+    <t>Tetrapropylammonium Borohydride</t>
+  </si>
+  <si>
+    <t>Tetramethylammonium Borohydride</t>
+  </si>
+  <si>
+    <t>Methylamine Borane</t>
+  </si>
+  <si>
+    <t>Butylamine Borane</t>
+  </si>
+  <si>
+    <t>Ethylamine Borane</t>
+  </si>
+  <si>
+    <t>Propylamine Borane</t>
+  </si>
+  <si>
+    <t>Trimethylbutylammonium borohydride</t>
+  </si>
+  <si>
+    <t>Tetrabutylphosphonium borohydride</t>
+  </si>
+  <si>
+    <t>Dimethylamine Borane</t>
+  </si>
+  <si>
+    <t>Trimethylamine Borane</t>
+  </si>
+  <si>
+    <t>[B-][NH2+]C</t>
+  </si>
+  <si>
+    <t>[B][N+](C)(C)C</t>
+  </si>
+  <si>
+    <t>[BH3-][NH2+]CCC</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t>CNC.[B]</t>
+  </si>
+  <si>
+    <t>CCN.[B]</t>
+  </si>
+  <si>
+    <t>CCCCN.[B]</t>
+  </si>
+  <si>
+    <t>[BH4-].[Li+]</t>
+  </si>
+  <si>
+    <t>[BH4-].[Na+]</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[BH4-]</t>
+  </si>
+  <si>
+    <t>CCCC[N+](CCCC)(CCCC)CCCC.[BH4-]</t>
+  </si>
+  <si>
+    <t>COCCOCCOC</t>
+  </si>
+  <si>
+    <t>COCCOCCOCCOC</t>
+  </si>
+  <si>
+    <t>COCCOCCOCCOCCOC</t>
+  </si>
+  <si>
+    <t>Thiourea</t>
+  </si>
+  <si>
+    <t>Thioacetamide</t>
+  </si>
+  <si>
+    <t>Thiobenzamide</t>
+  </si>
+  <si>
+    <t>Thioisonicotinamide</t>
+  </si>
+  <si>
+    <t>Pyrrole-2-thiocarboxamide</t>
+  </si>
+  <si>
+    <t>Pyridine-2-thiocarboxamide</t>
+  </si>
+  <si>
+    <t>Cyclopropanethiocarboxamide</t>
+  </si>
+  <si>
+    <t>C(=S)(N)N</t>
+  </si>
+  <si>
+    <t>CC(=S)N</t>
+  </si>
+  <si>
+    <t>C1=CC=C(C=C1)C(=S)N</t>
+  </si>
+  <si>
+    <t>Thioisobutyramide</t>
+  </si>
+  <si>
+    <t>C1=CN=CC=C1C(=S)N</t>
+  </si>
+  <si>
+    <t>CC(C)C(=S)N</t>
+  </si>
+  <si>
+    <t>C1=CNC(=C1)C(=S)N</t>
+  </si>
+  <si>
+    <t>C1=CC=NC(=C1)C(=S)N</t>
+  </si>
+  <si>
+    <t>C1CC1C(=S)N</t>
   </si>
 </sst>
 </file>
@@ -1296,18 +1464,12 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -1322,7 +1484,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1333,11 +1495,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1672,10 +1837,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3399CF41-2FA5-4790-AC55-DE65A2BCB50A}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
@@ -1803,137 +1968,446 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="6">
+        <f>(292+291+293+291.75)/4</f>
+        <v>291.9375</v>
+      </c>
+      <c r="E7" s="5">
+        <f>(18.303+18.285+18.28+18.476)/4*1000</f>
+        <v>18336</v>
+      </c>
+      <c r="F7" s="5">
+        <f>(-669.6-668.6)/2</f>
+        <v>-669.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5">
+        <v>284.2</v>
+      </c>
+      <c r="E8" s="5">
+        <v>21830</v>
+      </c>
+      <c r="F8" s="5">
+        <v>-63010</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="5">
+        <f>(209.1+209.15)/2</f>
+        <v>209.125</v>
+      </c>
+      <c r="E10" s="5">
+        <f>(17.78+17.795)/2*1000</f>
+        <v>17787.5</v>
+      </c>
+      <c r="F10" s="5">
+        <f>(-556.4-569.4)/2*1000</f>
+        <v>-562900</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="5">
+        <f>AVERAGE(228.15,228)</f>
+        <v>228.07499999999999</v>
+      </c>
+      <c r="E11" s="5">
+        <f>AVERAGE(23.71,23.715)*1000</f>
+        <v>23712.5</v>
+      </c>
+      <c r="F11" s="5">
+        <v>-687000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" s="5">
+        <v>243.45</v>
+      </c>
+      <c r="E12" s="5">
+        <v>29300</v>
+      </c>
+      <c r="F12" s="5">
+        <v>-814000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
+      <c r="C13" s="5"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="5">
+        <f>273.15+108</f>
+        <v>381.15</v>
+      </c>
+      <c r="E14" s="5">
+        <v>14600</v>
+      </c>
+      <c r="F14" s="5">
+        <v>-133400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="5">
+        <v>329.15</v>
+      </c>
+      <c r="E15" s="5">
+        <v>13800</v>
+      </c>
+      <c r="F15" s="5">
+        <v>-158000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="5">
+        <v>309.14999999999998</v>
+      </c>
+      <c r="E16" s="5">
+        <v>12100</v>
+      </c>
+      <c r="F16" s="5">
+        <v>-186000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="5">
+        <v>367.15</v>
+      </c>
+      <c r="E17" s="5">
+        <v>10500</v>
+      </c>
+      <c r="F17" s="5">
+        <v>-218000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="5">
+        <f>273.15+268</f>
+        <v>541.15</v>
+      </c>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5">
+        <v>-190800</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="5">
+        <v>673.15</v>
+      </c>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="5">
+      <c r="B28" s="5"/>
+      <c r="C28" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D28" s="5">
         <f>273.15+124</f>
         <v>397.15</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E28" s="5">
         <v>15800</v>
       </c>
-      <c r="F7" s="5"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5">
-        <f>(209.1+209.15)/2</f>
-        <v>209.125</v>
-      </c>
-      <c r="E8" s="5">
-        <f>(17.78+17.795)/2*1000</f>
-        <v>17787.5</v>
-      </c>
-      <c r="F8" s="5">
-        <f>(-556.4-569.4)/2*1000</f>
-        <v>-562900</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="6">
-        <f>(292+291+293+291.75)/4</f>
-        <v>291.9375</v>
-      </c>
-      <c r="E9">
-        <f>(18.303+18.285+18.28+18.476)/4*1000</f>
-        <v>18336</v>
-      </c>
-      <c r="F9">
-        <f>(-669.6-668.6)/2</f>
-        <v>-669.1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="5">
-        <v>284.2</v>
-      </c>
-      <c r="E10" s="5">
-        <v>21830</v>
-      </c>
-      <c r="F10" s="5">
-        <v>-63010</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="5">
-        <f>273.15+108</f>
-        <v>381.15</v>
-      </c>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5">
-        <v>-133400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="5">
-        <f>273.15+268</f>
-        <v>541.15</v>
-      </c>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5">
-        <v>-190800</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5">
-        <v>673.15</v>
-      </c>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="F28" s="5">
+        <v>-395000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C33" t="s">
+        <v>65</v>
+      </c>
+      <c r="D33">
+        <v>449.7</v>
+      </c>
+      <c r="E33">
+        <v>13597</v>
+      </c>
+      <c r="F33">
+        <v>-89100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C34" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34">
+        <v>385.7</v>
+      </c>
+      <c r="E34">
+        <v>18360</v>
+      </c>
+      <c r="F34">
+        <v>-73010</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35">
+        <v>387.15</v>
+      </c>
+      <c r="E35">
+        <v>17730</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36">
+        <v>473.15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D37" s="7">
+        <v>319.64999999999998</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C39" t="s">
+        <v>72</v>
+      </c>
+      <c r="D39">
+        <v>410.15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C40" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40">
+        <v>385.15</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1" xr:uid="{3399CF41-2FA5-4790-AC55-DE65A2BCB50A}">

</xml_diff>

<commit_message>
Initial attempt to use GP to predict activity coefficients. [PAUSED since HANNA exists]
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF32F9B-D4DF-4480-A69E-4D341762BCB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{684AAFCB-DA1C-43E3-A00B-A56D0AFEEF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
     <sheet name="CATALOG" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CATALOG!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -733,7 +734,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D22" authorId="0" shapeId="0" xr:uid="{63C390B0-F0DD-4E22-8006-4770ED582EEB}">
+    <comment ref="F22" authorId="0" shapeId="0" xr:uid="{E1A1E0C1-3AE1-4CDA-A225-D95E0807710C}">
       <text>
         <r>
           <rPr>
@@ -758,32 +759,55 @@
         </r>
       </text>
     </comment>
-    <comment ref="F22" authorId="0" shapeId="0" xr:uid="{E1A1E0C1-3AE1-4CDA-A225-D95E0807710C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D28" authorId="0" shapeId="0" xr:uid="{74CA7090-F16F-4E81-9C1D-4C76B0CA001F}">
+    <comment ref="D24" authorId="0" shapeId="0" xr:uid="{77977B3A-77FD-4B3F-B5BC-D929DC7D5296}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1)https://iris.unito.it/bitstream/2318/1995351/2/Dematteis%20-%20PhD%20Thesis%20-%20DEF_REFEREE.pdf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E24" authorId="0" shapeId="0" xr:uid="{569CA5D4-C30C-423C-827D-117707B91194}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1)https://iris.unito.it/bitstream/2318/1995351/2/Dematteis%20-%20PhD%20Thesis%20-%20DEF_REFEREE.pdf</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D29" authorId="0" shapeId="0" xr:uid="{74CA7090-F16F-4E81-9C1D-4C76B0CA001F}">
       <text>
         <r>
           <rPr>
@@ -805,6 +829,54 @@
           <t xml:space="preserve">
 Source(s):
 1)https://advanced.onlinelibrary.wiley.com/doi/10.1002/adma.202502566</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D34" authorId="0" shapeId="0" xr:uid="{D4CAD80C-B7CB-420F-8676-3A2ADB9B10C7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C1643192&amp;Mask=1EFF#Thermo-Gas</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E34" authorId="0" shapeId="0" xr:uid="{5850F739-EC51-4500-92CB-C367CCC5DCEE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+https://webbook.nist.gov/cgi/cbook.cgi?ID=C1643192&amp;Mask=1EFF#Thermo-Gas</t>
         </r>
       </text>
     </comment>
@@ -1192,7 +1264,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
   <si>
     <t>Full Name</t>
   </si>
@@ -1417,6 +1489,15 @@
   </si>
   <si>
     <t>C1CC1C(=S)N</t>
+  </si>
+  <si>
+    <t>Tetra-N-butylammonium bromide</t>
+  </si>
+  <si>
+    <t>Potassium Borohydride</t>
+  </si>
+  <si>
+    <t>[BH4-].[K+]</t>
   </si>
 </sst>
 </file>
@@ -1484,7 +1565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1495,14 +1576,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1837,7 +1912,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3399CF41-2FA5-4790-AC55-DE65A2BCB50A}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.28515625" bestFit="1" customWidth="1"/>
@@ -1949,463 +2024,441 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5" t="s">
+      <c r="C6" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6">
         <v>283.45999999999998</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6">
         <v>13800</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6">
         <v>-507500</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="6">
+      <c r="D7" s="4">
         <f>(292+291+293+291.75)/4</f>
         <v>291.9375</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7">
         <f>(18.303+18.285+18.28+18.476)/4*1000</f>
         <v>18336</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7">
         <f>(-669.6-668.6)/2</f>
         <v>-669.1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5" t="s">
+      <c r="C8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8">
         <v>284.2</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8">
         <v>21830</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8">
         <v>-63010</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-    </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10">
         <f>(209.1+209.15)/2</f>
         <v>209.125</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10">
         <f>(17.78+17.795)/2*1000</f>
         <v>17787.5</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10">
         <f>(-556.4-569.4)/2*1000</f>
         <v>-562900</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5" t="s">
+      <c r="C11" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11">
         <f>AVERAGE(228.15,228)</f>
         <v>228.07499999999999</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11">
         <f>AVERAGE(23.71,23.715)*1000</f>
         <v>23712.5</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11">
         <v>-687000</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5" t="s">
+      <c r="C12" t="s">
         <v>57</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12">
         <v>243.45</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12">
         <v>29300</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12">
         <v>-814000</v>
       </c>
     </row>
-    <row r="13" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="3"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5" t="s">
+      <c r="C14" t="s">
         <v>23</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14">
         <f>273.15+108</f>
         <v>381.15</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14">
         <v>14600</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14">
         <v>-133400</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5" t="s">
+      <c r="C15" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15">
         <v>329.15</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15">
         <v>13800</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15">
         <v>-158000</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+      <c r="A16" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5" t="s">
+      <c r="C16" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16">
         <v>309.14999999999998</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16">
         <v>12100</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16">
         <v>-186000</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+      <c r="A17" t="s">
         <v>43</v>
       </c>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5" t="s">
+      <c r="C17" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17">
         <v>367.15</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17">
         <v>10500</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17">
         <v>-218000</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5" t="s">
+      <c r="C18" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5" t="s">
+      <c r="C19" t="s">
         <v>46</v>
       </c>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5" t="s">
+      <c r="C20" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="4"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
+      <c r="A21" s="3"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5" t="s">
+      <c r="C22" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="5">
-        <f>273.15+268</f>
-        <v>541.15</v>
-      </c>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5">
+      <c r="D22">
+        <f>273.15+286</f>
+        <v>559.15</v>
+      </c>
+      <c r="E22">
+        <f>AVERAGE(7.56,6.72)*1000</f>
+        <v>7140</v>
+      </c>
+      <c r="F22">
         <v>-190800</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="4" t="s">
+      <c r="A23" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5" t="s">
+      <c r="C23" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23">
         <v>673.15</v>
       </c>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
+      <c r="E23">
+        <f>AVERAGE(16.9,15.1)*1000</f>
+        <v>16000</v>
+      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="4"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
+      <c r="A24" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24">
+        <f>273.15+605</f>
+        <v>878.15</v>
+      </c>
+      <c r="E24">
+        <f>AVERAGE(19.2)*1000</f>
+        <v>19200</v>
+      </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B25" s="5"/>
-      <c r="C25" s="5" t="s">
+      <c r="C26" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="5"/>
-      <c r="E25" s="5"/>
-      <c r="F25" s="5"/>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5" t="s">
+      <c r="C27" t="s">
         <v>31</v>
       </c>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="4" t="s">
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="9" t="s">
+      <c r="C28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5" t="s">
+      <c r="C29" t="s">
         <v>54</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D29">
         <f>273.15+124</f>
         <v>397.15</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E29">
         <v>15800</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F29">
         <v>-395000</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C31" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C32" s="5" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="3"/>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="5"/>
+      <c r="D34">
+        <v>395</v>
+      </c>
+      <c r="E34">
+        <v>16150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C36" t="s">
         <v>65</v>
       </c>
-      <c r="D33">
+      <c r="D36">
         <v>449.7</v>
       </c>
-      <c r="E33">
+      <c r="E36">
         <v>13597</v>
       </c>
-      <c r="F33">
+      <c r="F36">
         <v>-89100</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="4" t="s">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C37" t="s">
         <v>66</v>
       </c>
-      <c r="D34">
+      <c r="D37">
         <v>385.7</v>
       </c>
-      <c r="E34">
+      <c r="E37">
         <v>18360</v>
       </c>
-      <c r="F34">
+      <c r="F37">
         <v>-73010</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="4" t="s">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C38" t="s">
         <v>67</v>
       </c>
-      <c r="D35">
+      <c r="D38">
         <v>387.15</v>
       </c>
-      <c r="E35">
+      <c r="E38">
         <v>17730</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="4" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C36" t="s">
+      <c r="C39" t="s">
         <v>69</v>
       </c>
-      <c r="D36">
+      <c r="D39">
         <v>473.15</v>
       </c>
     </row>
-    <row r="37" spans="1:6" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="4" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C40" t="s">
         <v>70</v>
       </c>
-      <c r="D37" s="7">
+      <c r="D40">
         <v>319.64999999999998</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C38" t="s">
+      <c r="C41" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C39" t="s">
+      <c r="C42" t="s">
         <v>72</v>
       </c>
-      <c r="D39">
+      <c r="D42">
         <v>410.15</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C43" t="s">
         <v>73</v>
       </c>
-      <c r="D40">
+      <c r="D43">
         <v>385.15</v>
       </c>
     </row>
@@ -2434,7 +2487,7 @@
     <col min="6" max="6" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
IN PROGRESS - testing the predictive properties of the MTGPR given a small dataset
</commit_message>
<xml_diff>
--- a/data/input/pureComponents.xlsx
+++ b/data/input/pureComponents.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{684AAFCB-DA1C-43E3-A00B-A56D0AFEEF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91857889-0EA8-4489-B573-EC8153478EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{22E7D031-F429-4E0A-8A8B-4D129F5BB641}"/>
   </bookViews>
   <sheets>
-    <sheet name="CATALOG" sheetId="1" r:id="rId1"/>
+    <sheet name="Unfinished CATALOG" sheetId="1" r:id="rId1"/>
     <sheet name="Input" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">CATALOG!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Unfinished CATALOG'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>

</xml_diff>